<commit_message>
Update research notes and report labels
</commit_message>
<xml_diff>
--- a/outputs/cocoa-trading-v2/cocoa-trade-scenario.xlsx
+++ b/outputs/cocoa-trading-v2/cocoa-trade-scenario.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R8fb0d42195d8458d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trade Inputs" sheetId="2" r:id="R518b30f068474385"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario P&amp;L" sheetId="3" r:id="R5dbaf5e4212c4dcf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="4" r:id="Ref3fa7cc71cd43c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources Audit" sheetId="5" r:id="R09b306ea4158463c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R1325302a812744a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trade Inputs" sheetId="2" r:id="R023665ec5d4e4bcc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario P&amp;L" sheetId="3" r:id="R4957a7d16d274eb2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="4" r:id="Raa570e507ece40e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources Audit" sheetId="5" r:id="Rfb3c68bbc28c4644"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -684,7 +684,7 @@
         <x:color rgb="FF9B1C1C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDECEC"/>
         </x:patternFill>
       </x:fill>
@@ -695,7 +695,7 @@
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5E9"/>
         </x:patternFill>
       </x:fill>
@@ -706,7 +706,7 @@
         <x:color rgb="FF7C4A03"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4D6"/>
         </x:patternFill>
       </x:fill>
@@ -717,7 +717,7 @@
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5E9"/>
         </x:patternFill>
       </x:fill>
@@ -728,7 +728,7 @@
         <x:color rgb="FF9B1C1C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDECEC"/>
         </x:patternFill>
       </x:fill>
@@ -883,7 +883,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R130cc31923354629"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re71a6ea1ed1b4973"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1295,7 +1295,7 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="72" t="str">
-        <x:v>The workbook demonstrates instrument selection, capped-loss sizing and expiry scenarios. It deliberately does not claim executable pricing: replace the illustrative settlement, strikes and debit only with data your licence permits you to use.</x:v>
+        <x:v>The workbook documents instrument selection, capped-loss sizing and expiry scenarios. It does not claim executable pricing: replace the illustrative settlement, strikes and debit only with data your licence permits you to use.</x:v>
       </x:c>
       <x:c r="B16" s="73"/>
       <x:c r="C16" s="73"/>
@@ -2214,7 +2214,7 @@
     <x:mergeCell ref="A15:G17"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R989c9b8249a247b9"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0311f89871644513"/>
 </x:worksheet>
 </file>
 

</xml_diff>